<commit_message>
added skills page test cases
</commit_message>
<xml_diff>
--- a/testdata/ExData.xlsx
+++ b/testdata/ExData.xlsx
@@ -8,12 +8,13 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Pruthvi Raj\My projects\Playwright\OrangeHRM_POM_FRAMEWORK\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B789DDBC-D08D-4BD2-B3D8-37E2001B4D4F}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{B1ADA836-C318-46F1-B59B-004F9C68D177}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
+    <sheet name="Qualifications" sheetId="2" r:id="rId2"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -25,7 +26,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="18" uniqueCount="18">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="33">
   <si>
     <t>FirstName</t>
   </si>
@@ -79,6 +80,51 @@
   </si>
   <si>
     <t>Playwright5</t>
+  </si>
+  <si>
+    <t>SkillName</t>
+  </si>
+  <si>
+    <t>SkillDescription</t>
+  </si>
+  <si>
+    <t>EducationLevel</t>
+  </si>
+  <si>
+    <t>LicenceName</t>
+  </si>
+  <si>
+    <t>LanguageName</t>
+  </si>
+  <si>
+    <t>MembershipName</t>
+  </si>
+  <si>
+    <t>This is web automation tool</t>
+  </si>
+  <si>
+    <t>Play1</t>
+  </si>
+  <si>
+    <t>TypeScript1</t>
+  </si>
+  <si>
+    <t>VAGE1</t>
+  </si>
+  <si>
+    <t>Graduation1</t>
+  </si>
+  <si>
+    <t>Graduation2</t>
+  </si>
+  <si>
+    <t>VAGE2</t>
+  </si>
+  <si>
+    <t>TypeScript2</t>
+  </si>
+  <si>
+    <t>Play2</t>
   </si>
 </sst>
 </file>
@@ -495,4 +541,83 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet2.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{FF3AF2A5-692A-4A86-8EF4-085199F750F5}">
+  <dimension ref="A1:F3"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="10.90625" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="24.81640625" bestFit="1" customWidth="1"/>
+    <col min="3" max="3" width="13.90625" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="12.26953125" bestFit="1" customWidth="1"/>
+    <col min="5" max="5" width="14" bestFit="1" customWidth="1"/>
+    <col min="6" max="6" width="17" bestFit="1" customWidth="1"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A1" s="1" t="s">
+        <v>18</v>
+      </c>
+      <c r="B1" s="1" t="s">
+        <v>19</v>
+      </c>
+      <c r="C1" s="1" t="s">
+        <v>20</v>
+      </c>
+      <c r="D1" s="1" t="s">
+        <v>21</v>
+      </c>
+      <c r="E1" s="1" t="s">
+        <v>22</v>
+      </c>
+      <c r="F1" s="1" t="s">
+        <v>23</v>
+      </c>
+    </row>
+    <row r="2" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A2" t="s">
+        <v>9</v>
+      </c>
+      <c r="B2" t="s">
+        <v>24</v>
+      </c>
+      <c r="C2" t="s">
+        <v>28</v>
+      </c>
+      <c r="D2" t="s">
+        <v>27</v>
+      </c>
+      <c r="E2" t="s">
+        <v>26</v>
+      </c>
+      <c r="F2" t="s">
+        <v>25</v>
+      </c>
+    </row>
+    <row r="3" spans="1:6" x14ac:dyDescent="0.35">
+      <c r="A3" t="s">
+        <v>14</v>
+      </c>
+      <c r="B3" t="s">
+        <v>24</v>
+      </c>
+      <c r="C3" t="s">
+        <v>29</v>
+      </c>
+      <c r="D3" t="s">
+        <v>30</v>
+      </c>
+      <c r="E3" t="s">
+        <v>31</v>
+      </c>
+      <c r="F3" t="s">
+        <v>32</v>
+      </c>
+    </row>
+  </sheetData>
+  <phoneticPr fontId="2" type="noConversion"/>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>

<commit_message>
Added new test data for Jobs module
</commit_message>
<xml_diff>
--- a/testdata/ExData.xlsx
+++ b/testdata/ExData.xlsx
@@ -8,13 +8,14 @@
       <x15ac:absPath xmlns:x15ac="http://schemas.microsoft.com/office/spreadsheetml/2010/11/ac" url="E:\Pruthvi Raj\My projects\Playwright\OrangeHRM_POM_FRAMEWORK\testdata\"/>
     </mc:Choice>
   </mc:AlternateContent>
-  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{58A50319-5373-46D0-8CA5-D54C806ADFF0}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
+  <xr:revisionPtr revIDLastSave="0" documentId="13_ncr:1_{BE54A322-DBEA-4C04-87F0-582863A61623}" xr6:coauthVersionLast="47" xr6:coauthVersionMax="47" xr10:uidLastSave="{00000000-0000-0000-0000-000000000000}"/>
   <bookViews>
-    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="1" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
+    <workbookView xWindow="-110" yWindow="-110" windowWidth="19420" windowHeight="10300" activeTab="2" xr2:uid="{00000000-000D-0000-FFFF-FFFF00000000}"/>
   </bookViews>
   <sheets>
     <sheet name="Sheet1" sheetId="1" r:id="rId1"/>
     <sheet name="Qualifications" sheetId="2" r:id="rId2"/>
+    <sheet name="Job" sheetId="3" r:id="rId3"/>
   </sheets>
   <calcPr calcId="162913"/>
   <extLst>
@@ -26,7 +27,7 @@
 </file>
 
 <file path=xl/sharedStrings.xml><?xml version="1.0" encoding="utf-8"?>
-<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="36" uniqueCount="33">
+<sst xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" count="52" uniqueCount="49">
   <si>
     <t>FirstName</t>
   </si>
@@ -125,6 +126,54 @@
   </si>
   <si>
     <t>Play2</t>
+  </si>
+  <si>
+    <t>JobTitle</t>
+  </si>
+  <si>
+    <t>JobDescription</t>
+  </si>
+  <si>
+    <t>Note</t>
+  </si>
+  <si>
+    <t>PayGradeName</t>
+  </si>
+  <si>
+    <t>EmploymentStatusName</t>
+  </si>
+  <si>
+    <t>JobCategoryName</t>
+  </si>
+  <si>
+    <t>ShiftName</t>
+  </si>
+  <si>
+    <t>Playwright Automation</t>
+  </si>
+  <si>
+    <t>Need to Automate end to end work flows with positive and negative test cases</t>
+  </si>
+  <si>
+    <t>Need to have Typescript skill</t>
+  </si>
+  <si>
+    <t>Play Grade A</t>
+  </si>
+  <si>
+    <t>MinimumSalary</t>
+  </si>
+  <si>
+    <t>MaximumSalary</t>
+  </si>
+  <si>
+    <t>Permanent</t>
+  </si>
+  <si>
+    <t>SDET</t>
+  </si>
+  <si>
+    <t>UK Shift</t>
   </si>
 </sst>
 </file>
@@ -180,9 +229,18 @@
   <cellStyleXfs count="1">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0"/>
   </cellStyleXfs>
-  <cellXfs count="2">
+  <cellXfs count="5">
     <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0"/>
     <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1"/>
+    <xf numFmtId="0" fontId="1" fillId="2" borderId="0" xfId="0" applyFont="1" applyFill="1" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top"/>
+    </xf>
+    <xf numFmtId="0" fontId="0" fillId="0" borderId="0" xfId="0" applyAlignment="1">
+      <alignment horizontal="left" vertical="top" wrapText="1"/>
+    </xf>
   </cellXfs>
   <cellStyles count="1">
     <cellStyle name="Normal" xfId="0" builtinId="0"/>
@@ -620,4 +678,83 @@
   <phoneticPr fontId="2" type="noConversion"/>
   <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
 </worksheet>
+</file>
+
+<file path=xl/worksheets/sheet3.xml><?xml version="1.0" encoding="utf-8"?>
+<worksheet xmlns="http://schemas.openxmlformats.org/spreadsheetml/2006/main" xmlns:r="http://schemas.openxmlformats.org/officeDocument/2006/relationships" xmlns:mc="http://schemas.openxmlformats.org/markup-compatibility/2006" xmlns:x14ac="http://schemas.microsoft.com/office/spreadsheetml/2009/9/ac" xmlns:xr="http://schemas.microsoft.com/office/spreadsheetml/2014/revision" xmlns:xr2="http://schemas.microsoft.com/office/spreadsheetml/2015/revision2" xmlns:xr3="http://schemas.microsoft.com/office/spreadsheetml/2016/revision3" mc:Ignorable="x14ac xr xr2 xr3" xr:uid="{C538B7C3-455C-4DED-964C-3F9A48251BE0}">
+  <dimension ref="A1:I2"/>
+  <sheetFormatPr defaultRowHeight="14.5" x14ac:dyDescent="0.35"/>
+  <cols>
+    <col min="1" max="1" width="20" style="3" bestFit="1" customWidth="1"/>
+    <col min="2" max="2" width="34.54296875" style="3" customWidth="1"/>
+    <col min="3" max="3" width="24.6328125" style="3" bestFit="1" customWidth="1"/>
+    <col min="4" max="4" width="13.81640625" style="3" bestFit="1" customWidth="1"/>
+    <col min="5" max="6" width="13.81640625" style="3" customWidth="1"/>
+    <col min="7" max="7" width="21.6328125" style="3" bestFit="1" customWidth="1"/>
+    <col min="8" max="8" width="16" style="3" bestFit="1" customWidth="1"/>
+    <col min="9" max="9" width="9.453125" style="3" bestFit="1" customWidth="1"/>
+    <col min="10" max="16384" width="8.7265625" style="3"/>
+  </cols>
+  <sheetData>
+    <row r="1" spans="1:9" x14ac:dyDescent="0.35">
+      <c r="A1" s="2" t="s">
+        <v>33</v>
+      </c>
+      <c r="B1" s="2" t="s">
+        <v>34</v>
+      </c>
+      <c r="C1" s="2" t="s">
+        <v>35</v>
+      </c>
+      <c r="D1" s="2" t="s">
+        <v>36</v>
+      </c>
+      <c r="E1" s="2" t="s">
+        <v>44</v>
+      </c>
+      <c r="F1" s="2" t="s">
+        <v>45</v>
+      </c>
+      <c r="G1" s="2" t="s">
+        <v>37</v>
+      </c>
+      <c r="H1" s="2" t="s">
+        <v>38</v>
+      </c>
+      <c r="I1" s="2" t="s">
+        <v>39</v>
+      </c>
+    </row>
+    <row r="2" spans="1:9" ht="43.5" x14ac:dyDescent="0.35">
+      <c r="A2" s="3" t="s">
+        <v>40</v>
+      </c>
+      <c r="B2" s="4" t="s">
+        <v>41</v>
+      </c>
+      <c r="C2" s="3" t="s">
+        <v>42</v>
+      </c>
+      <c r="D2" s="3" t="s">
+        <v>43</v>
+      </c>
+      <c r="E2" s="3">
+        <v>50000</v>
+      </c>
+      <c r="F2" s="3">
+        <v>90000</v>
+      </c>
+      <c r="G2" s="3" t="s">
+        <v>46</v>
+      </c>
+      <c r="H2" s="3" t="s">
+        <v>47</v>
+      </c>
+      <c r="I2" s="3" t="s">
+        <v>48</v>
+      </c>
+    </row>
+  </sheetData>
+  <pageMargins left="0.7" right="0.7" top="0.75" bottom="0.75" header="0.3" footer="0.3"/>
+</worksheet>
 </file>
</xml_diff>